<commit_message>
changed the html report
</commit_message>
<xml_diff>
--- a/scans/pha.org.pk/reports/report.xlsx
+++ b/scans/pha.org.pk/reports/report.xlsx
@@ -17,7 +17,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Summary'!$A$1:$B$7</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Subdomains'!$A$1:$B$6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Live Hosts'!$A$1:$D$6</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Open Ports'!$A$1:$D$69</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Open Ports'!$A$1:$D$86</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Technologies'!$A$1:$C$6</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -504,7 +504,7 @@
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>68</v>
+        <v>85</v>
       </c>
     </row>
     <row r="6">
@@ -525,7 +525,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>12-08-2026</t>
+          <t>15-08-2026</t>
         </is>
       </c>
     </row>
@@ -566,7 +566,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>webmail.pha.org.pk</t>
+          <t>mail.pha.org.pk</t>
         </is>
       </c>
     </row>
@@ -576,7 +576,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>wildcard.pha.org.pk</t>
+          <t>mail2.pha.org.pk</t>
         </is>
       </c>
     </row>
@@ -586,7 +586,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>www.pha.org.pk</t>
+          <t>webmail.pha.org.pk</t>
         </is>
       </c>
     </row>
@@ -596,7 +596,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>mail.pha.org.pk</t>
+          <t>wildcard.pha.org.pk</t>
         </is>
       </c>
     </row>
@@ -606,7 +606,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>mail2.pha.org.pk</t>
+          <t>www.pha.org.pk</t>
         </is>
       </c>
     </row>
@@ -656,7 +656,7 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>https://webmail.pha.org.pk</t>
+          <t>https://wildcard.pha.org.pk</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr"/>
@@ -666,7 +666,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>https://mail.pha.org.pk</t>
+          <t>https://mail2.pha.org.pk</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr"/>
@@ -676,7 +676,7 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>https://wildcard.pha.org.pk</t>
+          <t>https://webmail.pha.org.pk</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr"/>
@@ -686,7 +686,7 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>http://www.pha.org.pk</t>
+          <t>https://mail.pha.org.pk</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr"/>
@@ -696,7 +696,7 @@
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>https://mail2.pha.org.pk</t>
+          <t>http://www.pha.org.pk</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr"/>
@@ -722,7 +722,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D69"/>
+  <dimension ref="A1:D86"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="21" customWidth="1" min="1" max="1"/>
@@ -756,7 +756,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>mail2.pha.org.pk</t>
+          <t>mail.pha.org.pk</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -778,7 +778,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>mail2.pha.org.pk</t>
+          <t>mail.pha.org.pk</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
@@ -800,7 +800,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>mail2.pha.org.pk</t>
+          <t>mail.pha.org.pk</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
@@ -822,7 +822,7 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>mail2.pha.org.pk</t>
+          <t>mail.pha.org.pk</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
@@ -844,7 +844,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>mail2.pha.org.pk</t>
+          <t>mail.pha.org.pk</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
@@ -866,7 +866,7 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>mail2.pha.org.pk</t>
+          <t>mail.pha.org.pk</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
@@ -888,7 +888,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>mail2.pha.org.pk</t>
+          <t>mail.pha.org.pk</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
@@ -910,7 +910,7 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>mail2.pha.org.pk</t>
+          <t>mail.pha.org.pk</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
@@ -932,7 +932,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>mail2.pha.org.pk</t>
+          <t>mail.pha.org.pk</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
@@ -947,14 +947,14 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>https; title=Softrack Technologies; server=Microsoft-IIS/10.0; status=303; redirect=https://mail2.pha.org.pk/login.php</t>
+          <t>https; title=Softrack Technologies; server=Microsoft-IIS/10.0; status=303; redirect=https://mail.pha.org.pk/login.php</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>mail2.pha.org.pk</t>
+          <t>mail.pha.org.pk</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
@@ -976,7 +976,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>mail2.pha.org.pk</t>
+          <t>mail.pha.org.pk</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
@@ -998,7 +998,7 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>mail2.pha.org.pk</t>
+          <t>mail.pha.org.pk</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
@@ -1020,7 +1020,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>mail2.pha.org.pk</t>
+          <t>mail.pha.org.pk</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
@@ -1042,7 +1042,7 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>mail2.pha.org.pk</t>
+          <t>mail.pha.org.pk</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
@@ -1064,7 +1064,7 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>mail2.pha.org.pk</t>
+          <t>mail.pha.org.pk</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
@@ -1086,7 +1086,7 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>mail2.pha.org.pk</t>
+          <t>mail.pha.org.pk</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
@@ -1108,7 +1108,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>mail2.pha.org.pk</t>
+          <t>mail.pha.org.pk</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
@@ -1130,7 +1130,7 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>webmail.pha.org.pk</t>
+          <t>mail2.pha.org.pk</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
@@ -1152,7 +1152,7 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>webmail.pha.org.pk</t>
+          <t>mail2.pha.org.pk</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
@@ -1174,7 +1174,7 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>webmail.pha.org.pk</t>
+          <t>mail2.pha.org.pk</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
@@ -1196,7 +1196,7 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>webmail.pha.org.pk</t>
+          <t>mail2.pha.org.pk</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
@@ -1211,14 +1211,14 @@
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>http; title=MailEnable Web Mail; server=Microsoft-IIS/10.0; status=301; redirect=https://webmail.pha.org.pk/</t>
+          <t>http; title=Web Server's Default Page; server=Microsoft-IIS/10.0; status=200</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>webmail.pha.org.pk</t>
+          <t>mail2.pha.org.pk</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
@@ -1240,7 +1240,7 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>webmail.pha.org.pk</t>
+          <t>mail2.pha.org.pk</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
@@ -1262,7 +1262,7 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>webmail.pha.org.pk</t>
+          <t>mail2.pha.org.pk</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
@@ -1284,7 +1284,7 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>webmail.pha.org.pk</t>
+          <t>mail2.pha.org.pk</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
@@ -1306,7 +1306,7 @@
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>webmail.pha.org.pk</t>
+          <t>mail2.pha.org.pk</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
@@ -1321,14 +1321,14 @@
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>https; title=MailEnable Web Mail; server=Microsoft-IIS/10.0; status=302; redirect=/Mondo/lang/sys/login.aspx</t>
+          <t>https; title=Softrack Technologies; server=Microsoft-IIS/10.0; status=303; redirect=https://mail2.pha.org.pk/login.php</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>webmail.pha.org.pk</t>
+          <t>mail2.pha.org.pk</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
@@ -1350,7 +1350,7 @@
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>webmail.pha.org.pk</t>
+          <t>mail2.pha.org.pk</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
@@ -1372,7 +1372,7 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>webmail.pha.org.pk</t>
+          <t>mail2.pha.org.pk</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
@@ -1394,7 +1394,7 @@
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>webmail.pha.org.pk</t>
+          <t>mail2.pha.org.pk</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
@@ -1416,7 +1416,7 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>webmail.pha.org.pk</t>
+          <t>mail2.pha.org.pk</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
@@ -1438,7 +1438,7 @@
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>webmail.pha.org.pk</t>
+          <t>mail2.pha.org.pk</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
@@ -1460,7 +1460,7 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>webmail.pha.org.pk</t>
+          <t>mail2.pha.org.pk</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
@@ -1482,7 +1482,7 @@
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>webmail.pha.org.pk</t>
+          <t>mail2.pha.org.pk</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
@@ -1504,7 +1504,7 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>wildcard.pha.org.pk</t>
+          <t>webmail.pha.org.pk</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
@@ -1526,7 +1526,7 @@
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>wildcard.pha.org.pk</t>
+          <t>webmail.pha.org.pk</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
@@ -1548,7 +1548,7 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>wildcard.pha.org.pk</t>
+          <t>webmail.pha.org.pk</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
@@ -1570,7 +1570,7 @@
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>wildcard.pha.org.pk</t>
+          <t>webmail.pha.org.pk</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
@@ -1585,14 +1585,14 @@
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>http; title=Web Server's Default Page; server=Microsoft-IIS/10.0; status=200</t>
+          <t>http; title=MailEnable Web Mail; server=Microsoft-IIS/10.0; status=301; redirect=https://webmail.pha.org.pk/</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>wildcard.pha.org.pk</t>
+          <t>webmail.pha.org.pk</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
@@ -1614,7 +1614,7 @@
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>wildcard.pha.org.pk</t>
+          <t>webmail.pha.org.pk</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
@@ -1636,7 +1636,7 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>wildcard.pha.org.pk</t>
+          <t>webmail.pha.org.pk</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
@@ -1658,7 +1658,7 @@
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>wildcard.pha.org.pk</t>
+          <t>webmail.pha.org.pk</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
@@ -1680,7 +1680,7 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>wildcard.pha.org.pk</t>
+          <t>webmail.pha.org.pk</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
@@ -1695,14 +1695,14 @@
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>https; title=Softrack Technologies; server=Microsoft-IIS/10.0; status=303; redirect=https://wildcard.pha.org.pk/login.php</t>
+          <t>https; title=MailEnable Web Mail; server=Microsoft-IIS/10.0; status=302; redirect=/Mondo/lang/sys/login.aspx</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>wildcard.pha.org.pk</t>
+          <t>webmail.pha.org.pk</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
@@ -1724,7 +1724,7 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>wildcard.pha.org.pk</t>
+          <t>webmail.pha.org.pk</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
@@ -1746,7 +1746,7 @@
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>wildcard.pha.org.pk</t>
+          <t>webmail.pha.org.pk</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
@@ -1768,7 +1768,7 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>wildcard.pha.org.pk</t>
+          <t>webmail.pha.org.pk</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
@@ -1790,7 +1790,7 @@
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>wildcard.pha.org.pk</t>
+          <t>webmail.pha.org.pk</t>
         </is>
       </c>
       <c r="B49" s="2" t="inlineStr">
@@ -1812,7 +1812,7 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>wildcard.pha.org.pk</t>
+          <t>webmail.pha.org.pk</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
@@ -1834,7 +1834,7 @@
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>wildcard.pha.org.pk</t>
+          <t>webmail.pha.org.pk</t>
         </is>
       </c>
       <c r="B51" s="2" t="inlineStr">
@@ -1856,7 +1856,7 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>wildcard.pha.org.pk</t>
+          <t>webmail.pha.org.pk</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
@@ -1878,7 +1878,7 @@
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>www.pha.org.pk</t>
+          <t>wildcard.pha.org.pk</t>
         </is>
       </c>
       <c r="B53" s="2" t="inlineStr">
@@ -1900,7 +1900,7 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>www.pha.org.pk</t>
+          <t>wildcard.pha.org.pk</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
@@ -1922,7 +1922,7 @@
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>www.pha.org.pk</t>
+          <t>wildcard.pha.org.pk</t>
         </is>
       </c>
       <c r="B55" s="2" t="inlineStr">
@@ -1944,7 +1944,7 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>www.pha.org.pk</t>
+          <t>wildcard.pha.org.pk</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr">
@@ -1959,14 +1959,14 @@
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>http; title=Pakistan Hotels Association | Welcome to PHA...; server=Microsoft-IIS/10.0; status=301; redirect=https://www.pha.org.pk/</t>
+          <t>http; title=Web Server's Default Page; server=Microsoft-IIS/10.0; status=200</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>www.pha.org.pk</t>
+          <t>wildcard.pha.org.pk</t>
         </is>
       </c>
       <c r="B57" s="2" t="inlineStr">
@@ -1988,7 +1988,7 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>www.pha.org.pk</t>
+          <t>wildcard.pha.org.pk</t>
         </is>
       </c>
       <c r="B58" s="2" t="inlineStr">
@@ -2010,7 +2010,7 @@
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>www.pha.org.pk</t>
+          <t>wildcard.pha.org.pk</t>
         </is>
       </c>
       <c r="B59" s="2" t="inlineStr">
@@ -2032,7 +2032,7 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>www.pha.org.pk</t>
+          <t>wildcard.pha.org.pk</t>
         </is>
       </c>
       <c r="B60" s="2" t="inlineStr">
@@ -2054,7 +2054,7 @@
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>www.pha.org.pk</t>
+          <t>wildcard.pha.org.pk</t>
         </is>
       </c>
       <c r="B61" s="2" t="inlineStr">
@@ -2069,14 +2069,14 @@
       </c>
       <c r="D61" s="2" t="inlineStr">
         <is>
-          <t>https; title=Pakistan Hotels Association | Welcome to PHA...; server=Microsoft-IIS/10.0; status=200</t>
+          <t>https; title=Softrack Technologies; server=Microsoft-IIS/10.0; status=303; redirect=https://wildcard.pha.org.pk/login.php</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>www.pha.org.pk</t>
+          <t>wildcard.pha.org.pk</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
@@ -2098,7 +2098,7 @@
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>www.pha.org.pk</t>
+          <t>wildcard.pha.org.pk</t>
         </is>
       </c>
       <c r="B63" s="2" t="inlineStr">
@@ -2120,7 +2120,7 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>www.pha.org.pk</t>
+          <t>wildcard.pha.org.pk</t>
         </is>
       </c>
       <c r="B64" s="2" t="inlineStr">
@@ -2142,7 +2142,7 @@
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>www.pha.org.pk</t>
+          <t>wildcard.pha.org.pk</t>
         </is>
       </c>
       <c r="B65" s="2" t="inlineStr">
@@ -2164,7 +2164,7 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>www.pha.org.pk</t>
+          <t>wildcard.pha.org.pk</t>
         </is>
       </c>
       <c r="B66" s="2" t="inlineStr">
@@ -2186,7 +2186,7 @@
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>www.pha.org.pk</t>
+          <t>wildcard.pha.org.pk</t>
         </is>
       </c>
       <c r="B67" s="2" t="inlineStr">
@@ -2208,7 +2208,7 @@
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>www.pha.org.pk</t>
+          <t>wildcard.pha.org.pk</t>
         </is>
       </c>
       <c r="B68" s="2" t="inlineStr">
@@ -2230,27 +2230,401 @@
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
         <is>
+          <t>wildcard.pha.org.pk</t>
+        </is>
+      </c>
+      <c r="B69" s="2" t="inlineStr">
+        <is>
+          <t>8443</t>
+        </is>
+      </c>
+      <c r="C69" s="2" t="inlineStr">
+        <is>
+          <t>TCP</t>
+        </is>
+      </c>
+      <c r="D69" s="2" t="inlineStr">
+        <is>
+          <t>pcsync-https</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="inlineStr">
+        <is>
           <t>www.pha.org.pk</t>
         </is>
       </c>
-      <c r="B69" s="2" t="inlineStr">
+      <c r="B70" s="2" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="C70" s="2" t="inlineStr">
+        <is>
+          <t>TCP</t>
+        </is>
+      </c>
+      <c r="D70" s="2" t="inlineStr">
+        <is>
+          <t>ftp</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="2" t="inlineStr">
+        <is>
+          <t>www.pha.org.pk</t>
+        </is>
+      </c>
+      <c r="B71" s="2" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="C71" s="2" t="inlineStr">
+        <is>
+          <t>TCP</t>
+        </is>
+      </c>
+      <c r="D71" s="2" t="inlineStr">
+        <is>
+          <t>smtp</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="2" t="inlineStr">
+        <is>
+          <t>www.pha.org.pk</t>
+        </is>
+      </c>
+      <c r="B72" s="2" t="inlineStr">
+        <is>
+          <t>53</t>
+        </is>
+      </c>
+      <c r="C72" s="2" t="inlineStr">
+        <is>
+          <t>TCP</t>
+        </is>
+      </c>
+      <c r="D72" s="2" t="inlineStr">
+        <is>
+          <t>domain</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="2" t="inlineStr">
+        <is>
+          <t>www.pha.org.pk</t>
+        </is>
+      </c>
+      <c r="B73" s="2" t="inlineStr">
+        <is>
+          <t>80</t>
+        </is>
+      </c>
+      <c r="C73" s="2" t="inlineStr">
+        <is>
+          <t>TCP</t>
+        </is>
+      </c>
+      <c r="D73" s="2" t="inlineStr">
+        <is>
+          <t>http; title=Pakistan Hotels Association | Welcome to PHA...; server=Microsoft-IIS/10.0; status=301; redirect=https://www.pha.org.pk/</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="2" t="inlineStr">
+        <is>
+          <t>www.pha.org.pk</t>
+        </is>
+      </c>
+      <c r="B74" s="2" t="inlineStr">
+        <is>
+          <t>110</t>
+        </is>
+      </c>
+      <c r="C74" s="2" t="inlineStr">
+        <is>
+          <t>TCP</t>
+        </is>
+      </c>
+      <c r="D74" s="2" t="inlineStr">
+        <is>
+          <t>pop3</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="2" t="inlineStr">
+        <is>
+          <t>www.pha.org.pk</t>
+        </is>
+      </c>
+      <c r="B75" s="2" t="inlineStr">
+        <is>
+          <t>135</t>
+        </is>
+      </c>
+      <c r="C75" s="2" t="inlineStr">
+        <is>
+          <t>TCP</t>
+        </is>
+      </c>
+      <c r="D75" s="2" t="inlineStr">
+        <is>
+          <t>epmap</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="2" t="inlineStr">
+        <is>
+          <t>www.pha.org.pk</t>
+        </is>
+      </c>
+      <c r="B76" s="2" t="inlineStr">
+        <is>
+          <t>139</t>
+        </is>
+      </c>
+      <c r="C76" s="2" t="inlineStr">
+        <is>
+          <t>TCP</t>
+        </is>
+      </c>
+      <c r="D76" s="2" t="inlineStr">
+        <is>
+          <t>netbios-ssn</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="2" t="inlineStr">
+        <is>
+          <t>www.pha.org.pk</t>
+        </is>
+      </c>
+      <c r="B77" s="2" t="inlineStr">
+        <is>
+          <t>143</t>
+        </is>
+      </c>
+      <c r="C77" s="2" t="inlineStr">
+        <is>
+          <t>TCP</t>
+        </is>
+      </c>
+      <c r="D77" s="2" t="inlineStr">
+        <is>
+          <t>imap</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="2" t="inlineStr">
+        <is>
+          <t>www.pha.org.pk</t>
+        </is>
+      </c>
+      <c r="B78" s="2" t="inlineStr">
+        <is>
+          <t>443</t>
+        </is>
+      </c>
+      <c r="C78" s="2" t="inlineStr">
+        <is>
+          <t>TCP</t>
+        </is>
+      </c>
+      <c r="D78" s="2" t="inlineStr">
+        <is>
+          <t>https; title=Pakistan Hotels Association | Welcome to PHA...; server=Microsoft-IIS/10.0; status=200</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="2" t="inlineStr">
+        <is>
+          <t>www.pha.org.pk</t>
+        </is>
+      </c>
+      <c r="B79" s="2" t="inlineStr">
+        <is>
+          <t>445</t>
+        </is>
+      </c>
+      <c r="C79" s="2" t="inlineStr">
+        <is>
+          <t>TCP</t>
+        </is>
+      </c>
+      <c r="D79" s="2" t="inlineStr">
+        <is>
+          <t>microsoft-ds</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="2" t="inlineStr">
+        <is>
+          <t>www.pha.org.pk</t>
+        </is>
+      </c>
+      <c r="B80" s="2" t="inlineStr">
+        <is>
+          <t>465</t>
+        </is>
+      </c>
+      <c r="C80" s="2" t="inlineStr">
+        <is>
+          <t>TCP</t>
+        </is>
+      </c>
+      <c r="D80" s="2" t="inlineStr">
+        <is>
+          <t>urd</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="2" t="inlineStr">
+        <is>
+          <t>www.pha.org.pk</t>
+        </is>
+      </c>
+      <c r="B81" s="2" t="inlineStr">
+        <is>
+          <t>587</t>
+        </is>
+      </c>
+      <c r="C81" s="2" t="inlineStr">
+        <is>
+          <t>TCP</t>
+        </is>
+      </c>
+      <c r="D81" s="2" t="inlineStr">
+        <is>
+          <t>submission</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="inlineStr">
+        <is>
+          <t>www.pha.org.pk</t>
+        </is>
+      </c>
+      <c r="B82" s="2" t="inlineStr">
+        <is>
+          <t>993</t>
+        </is>
+      </c>
+      <c r="C82" s="2" t="inlineStr">
+        <is>
+          <t>TCP</t>
+        </is>
+      </c>
+      <c r="D82" s="2" t="inlineStr">
+        <is>
+          <t>imaps</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="2" t="inlineStr">
+        <is>
+          <t>www.pha.org.pk</t>
+        </is>
+      </c>
+      <c r="B83" s="2" t="inlineStr">
+        <is>
+          <t>995</t>
+        </is>
+      </c>
+      <c r="C83" s="2" t="inlineStr">
+        <is>
+          <t>TCP</t>
+        </is>
+      </c>
+      <c r="D83" s="2" t="inlineStr">
+        <is>
+          <t>pop3s</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="2" t="inlineStr">
+        <is>
+          <t>www.pha.org.pk</t>
+        </is>
+      </c>
+      <c r="B84" s="2" t="inlineStr">
+        <is>
+          <t>1433</t>
+        </is>
+      </c>
+      <c r="C84" s="2" t="inlineStr">
+        <is>
+          <t>TCP</t>
+        </is>
+      </c>
+      <c r="D84" s="2" t="inlineStr">
+        <is>
+          <t>ms-sql-s</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="2" t="inlineStr">
+        <is>
+          <t>www.pha.org.pk</t>
+        </is>
+      </c>
+      <c r="B85" s="2" t="inlineStr">
+        <is>
+          <t>3389</t>
+        </is>
+      </c>
+      <c r="C85" s="2" t="inlineStr">
+        <is>
+          <t>TCP</t>
+        </is>
+      </c>
+      <c r="D85" s="2" t="inlineStr">
+        <is>
+          <t>ms-wbt-server</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="2" t="inlineStr">
+        <is>
+          <t>www.pha.org.pk</t>
+        </is>
+      </c>
+      <c r="B86" s="2" t="inlineStr">
         <is>
           <t>8443</t>
         </is>
       </c>
-      <c r="C69" s="2" t="inlineStr">
-        <is>
-          <t>TCP</t>
-        </is>
-      </c>
-      <c r="D69" s="2" t="inlineStr">
+      <c r="C86" s="2" t="inlineStr">
+        <is>
+          <t>TCP</t>
+        </is>
+      </c>
+      <c r="D86" s="2" t="inlineStr">
         <is>
           <t>pcsync-https</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D69"/>
+  <autoFilter ref="A1:D86"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2265,7 +2639,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
-    <col width="31" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
     <col width="9" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
@@ -2289,12 +2663,12 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>https://webmail.pha.org.pk</t>
+          <t>https://wildcard.pha.org.pk</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>HTTPX: HTML5</t>
+          <t>HTTPX: unreachable</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr"/>
@@ -2302,12 +2676,12 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>https://mail.pha.org.pk</t>
+          <t>https://mail2.pha.org.pk</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>HTTPX: no fingerprint matched</t>
+          <t>HTTPX: unreachable</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr"/>
@@ -2315,12 +2689,12 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>https://wildcard.pha.org.pk</t>
+          <t>https://webmail.pha.org.pk</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>HTTPX: no fingerprint matched</t>
+          <t>HTTPX: HTML5</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr"/>
@@ -2328,12 +2702,12 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>http://www.pha.org.pk</t>
+          <t>https://mail.pha.org.pk</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>HTTPX: HTML5</t>
+          <t>HTTPX: unreachable</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr"/>
@@ -2341,12 +2715,12 @@
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>https://mail2.pha.org.pk</t>
+          <t>http://www.pha.org.pk</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>HTTPX: no fingerprint matched</t>
+          <t>HTTPX: HTML5</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr"/>

</xml_diff>